<commit_message>
feat: add New API listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2525,32 +2525,62 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="0" t="n">
         <v>51</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="0" t="inlineStr">
         <is>
           <t>sudoflow</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>https://sudoflow.top/sign-up?aff=WLW8</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>GPT</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="0" t="inlineStr">
         <is>
           <t>AFF：https://sudoflow.top/sign-up?aff=WLW8 注册：QQ邮箱注册 倍率：0.065x的gpt 邀请：注册送7 刀</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="0" t="inlineStr">
         <is>
           <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>52</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>New API</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://xxs.l.cd/sign-up?aff=RhO4</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>注册赠送;DeepSeek</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>注册送 50，只有 DeepSeek 可用</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>

</xml_diff>